<commit_message>
Rebuild answer workbooks Q11-90 with per-part highlights; embeds for bank Q3-Q10
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/practice/answers/s1_q08.xlsx
+++ b/practice/answers/s1_q08.xlsx
@@ -1,69 +1,133 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
   <workbookPr/>
-  <workbookProtection/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_884D7FDFD678FC5FEC7F0C35456D1E78B0D4EDCB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DA07BD7-00FA-4C24-906B-BBE1FD9CABCB}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Answer" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+  <si>
+    <t>Rate ($/tonne)</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Tonnes</t>
+  </si>
+  <si>
+    <t>Trucking cost</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>AVERAGE of cost column</t>
+  </si>
+  <si>
+    <t>Total cost / COUNT</t>
+  </si>
+  <si>
+    <t>Total at $11.90 rate</t>
+  </si>
+  <si>
+    <t>With 12.75 typed into every row, changing the rate means finding and editing five separate formulas. Miss one and the sheet is wrong with no warning -- the total still looks plausible. Pointing every row at the one rate cell makes the change a single edit.</t>
+  </si>
+  <si>
+    <t>Part (a)</t>
+  </si>
+  <si>
+    <t>Part (b)</t>
+  </si>
+  <si>
+    <t>Part (c)</t>
+  </si>
+  <si>
+    <t>Part (d)</t>
+  </si>
+  <si>
+    <t>Part (e)</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="166" formatCode="DD-MMM-YY"/>
+    <numFmt numFmtId="166" formatCode="dd\-mmm\-yy"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
   <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="7">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
+        <fgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CFE2F3"/>
+        <fgColor rgb="FFCFE2F3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
+        <fgColor rgb="FFF4CCCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D2E9"/>
+        <fgColor rgb="FFD9D2E9"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,100 +143,42 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="19">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -460,222 +466,187 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col min="1" max="1" width="21" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Rate ($/tonne)</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2">
         <v>12.75</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>Tonnes</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Trucking cost</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
+    <row r="3" spans="1:7">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="4">
         <v>46277</v>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="5">
         <v>28.4</v>
       </c>
       <c r="C4" s="6">
         <f>B4*$B$1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
+        <v>362.09999999999997</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="4">
         <v>46284</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="5">
         <v>31.7</v>
       </c>
       <c r="C5" s="6">
         <f>B5*$B$1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+        <v>404.17500000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="4">
         <v>46291</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="5">
         <v>26.9</v>
       </c>
       <c r="C6" s="6">
         <f>B6*$B$1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
+        <v>342.97499999999997</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="4">
         <v>46298</v>
       </c>
-      <c r="B7" s="5" t="n">
-        <v>34.2</v>
+      <c r="B7" s="5">
+        <v>34.200000000000003</v>
       </c>
       <c r="C7" s="6">
         <f>B7*$B$1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+        <v>436.05</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="4">
         <v>46305</v>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="5">
         <v>29.8</v>
       </c>
       <c r="C8" s="6">
         <f>B8*$B$1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
+        <v>379.95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="7" t="s">
+        <v>4</v>
       </c>
       <c r="B9" s="8">
         <f>SUM(B4:B8)</f>
-        <v/>
+        <v>151</v>
       </c>
       <c r="C9" s="9">
         <f>SUM(C4:C8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>AVERAGE of cost column</t>
-        </is>
+        <v>1925.25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="10" t="s">
+        <v>5</v>
       </c>
       <c r="B11" s="11">
         <f>AVERAGE(C4:C8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>Total cost / COUNT</t>
-        </is>
+        <v>385.05</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="10" t="s">
+        <v>6</v>
       </c>
       <c r="B12" s="11">
         <f>C9/COUNT(B4:B8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Total at $11.90 rate</t>
-        </is>
+        <v>385.05</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="12" t="s">
+        <v>7</v>
       </c>
       <c r="B13" s="13">
         <f>B9*11.9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="14" t="inlineStr">
-        <is>
-          <t>With 12.75 typed into every row, changing the rate means finding and editing five separate formulas. Miss one and the sheet is wrong with no warning -- the total still looks plausible. Pointing every row at the one rate cell makes the change a single edit.</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="n"/>
-      <c r="C15" s="15" t="n"/>
-      <c r="D15" s="15" t="n"/>
-      <c r="E15" s="15" t="n"/>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="15" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="n"/>
-      <c r="B16" s="15" t="n"/>
-      <c r="C16" s="15" t="n"/>
-      <c r="D16" s="15" t="n"/>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="15" t="n"/>
-      <c r="G16" s="15" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="n"/>
-      <c r="B17" s="15" t="n"/>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="15" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="15" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>Part (a)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="17" t="inlineStr">
-        <is>
-          <t>Part (b)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>Part (c)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>Part (d)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>Part (e)</t>
-        </is>
+        <v>1796.9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="18"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="18"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="14" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>